<commit_message>
📊 Deploy Selenium E2E Reports — Build #3 2fc69e376d1558b77f7516ed34e4927a29622489
</commit_message>
<xml_diff>
--- a/reports/latest/reports/Excel/Execution_Summary.xlsx
+++ b/reports/latest/reports/Excel/Execution_Summary.xlsx
@@ -484,7 +484,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -492,7 +492,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>